<commit_message>
All results with zoom aug
</commit_message>
<xml_diff>
--- a/Results/Tables/Confusion_Matrices/All_Train_Confusion_Matrices.xlsx
+++ b/Results/Tables/Confusion_Matrices/All_Train_Confusion_Matrices.xlsx
@@ -410,21 +410,21 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>68</v>
-      </c>
-      <c r="C2">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3">
-        <v>43</v>
-      </c>
-      <c r="C3">
-        <v>53</v>
+        <v>451</v>
+      </c>
+      <c r="C2">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3">
+        <v>444</v>
+      </c>
+      <c r="C3">
+        <v>196</v>
       </c>
     </row>
   </sheetData>
@@ -450,21 +450,21 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>0</v>
-      </c>
-      <c r="C2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3">
-        <v>0</v>
-      </c>
-      <c r="C3">
-        <v>0</v>
+        <v>475</v>
+      </c>
+      <c r="C2">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3">
+        <v>412</v>
+      </c>
+      <c r="C3">
+        <v>228</v>
       </c>
     </row>
   </sheetData>
@@ -490,21 +490,21 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>159</v>
-      </c>
-      <c r="C2">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3">
-        <v>139</v>
-      </c>
-      <c r="C3">
-        <v>181</v>
+        <v>495</v>
+      </c>
+      <c r="C2">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3">
+        <v>435</v>
+      </c>
+      <c r="C3">
+        <v>205</v>
       </c>
     </row>
   </sheetData>
@@ -530,21 +530,21 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>526</v>
-      </c>
-      <c r="C2">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3">
-        <v>541</v>
-      </c>
-      <c r="C3">
-        <v>99</v>
+        <v>581</v>
+      </c>
+      <c r="C2">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3">
+        <v>518</v>
+      </c>
+      <c r="C3">
+        <v>122</v>
       </c>
     </row>
   </sheetData>
@@ -570,21 +570,21 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>0</v>
-      </c>
-      <c r="C2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3">
-        <v>0</v>
-      </c>
-      <c r="C3">
-        <v>0</v>
+        <v>288</v>
+      </c>
+      <c r="C2">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3">
+        <v>288</v>
+      </c>
+      <c r="C3">
+        <v>352</v>
       </c>
     </row>
   </sheetData>
@@ -610,21 +610,21 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>0</v>
-      </c>
-      <c r="C2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3">
-        <v>0</v>
-      </c>
-      <c r="C3">
-        <v>0</v>
+        <v>352</v>
+      </c>
+      <c r="C2">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3">
+        <v>352</v>
+      </c>
+      <c r="C3">
+        <v>288</v>
       </c>
     </row>
   </sheetData>
@@ -650,21 +650,21 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>0</v>
-      </c>
-      <c r="C2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3">
-        <v>0</v>
-      </c>
-      <c r="C3">
-        <v>0</v>
+        <v>566</v>
+      </c>
+      <c r="C2">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3">
+        <v>509</v>
+      </c>
+      <c r="C3">
+        <v>131</v>
       </c>
     </row>
   </sheetData>
@@ -690,21 +690,21 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>199</v>
-      </c>
-      <c r="C2">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3">
-        <v>159</v>
-      </c>
-      <c r="C3">
-        <v>161</v>
+        <v>586</v>
+      </c>
+      <c r="C2">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3">
+        <v>567</v>
+      </c>
+      <c r="C3">
+        <v>73</v>
       </c>
     </row>
   </sheetData>
@@ -730,21 +730,21 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>10</v>
-      </c>
-      <c r="C2">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3">
-        <v>4</v>
-      </c>
-      <c r="C3">
-        <v>92</v>
+        <v>451</v>
+      </c>
+      <c r="C2">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3">
+        <v>421</v>
+      </c>
+      <c r="C3">
+        <v>219</v>
       </c>
     </row>
   </sheetData>
@@ -770,21 +770,21 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>91</v>
-      </c>
-      <c r="C2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3">
-        <v>49</v>
-      </c>
-      <c r="C3">
-        <v>47</v>
+        <v>503</v>
+      </c>
+      <c r="C2">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3">
+        <v>473</v>
+      </c>
+      <c r="C3">
+        <v>167</v>
       </c>
     </row>
   </sheetData>
@@ -810,21 +810,21 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>0</v>
-      </c>
-      <c r="C2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3">
-        <v>0</v>
-      </c>
-      <c r="C3">
-        <v>0</v>
+        <v>559</v>
+      </c>
+      <c r="C2">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3">
+        <v>507</v>
+      </c>
+      <c r="C3">
+        <v>133</v>
       </c>
     </row>
   </sheetData>
@@ -850,21 +850,21 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>0</v>
-      </c>
-      <c r="C2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3">
-        <v>0</v>
-      </c>
-      <c r="C3">
-        <v>0</v>
+        <v>491</v>
+      </c>
+      <c r="C2">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3">
+        <v>461</v>
+      </c>
+      <c r="C3">
+        <v>179</v>
       </c>
     </row>
   </sheetData>

</xml_diff>